<commit_message>
Prepare for the public release and the Zenodo archive
- CITATION.cff and .zenodo.json, so the Zenodo record carries the paper's title
  and the four authors with affiliations rather than the repository name and
  GitHub usernames, which is what it defaults to.
- docs/AlloQuant_output_file_manifest_v7r3: experiment.csv was listed as a
  Module 1 output. It is a user-supplied input. Nothing in the pipeline writes
  it, and run_kinase_pipeline_v7r3.py deliberately omits it from
  DEFAULT_OUTPUT_FILES so archiving cannot destroy the user's design file.
  Stage is now "User input" and the preamble no longer claims Module 1 writes
  every file in the table.
- data/README.md: the main figure numbers were remapped in the manuscript so
  that Results cites them in ascending order. The structural handshake figure
  is now Fig 4, SRC autophosphorylation Fig 5, spine coupling Fig 6.

Assisted-by: Claude Opus 5 (Anthropic)
</commit_message>
<xml_diff>
--- a/docs/AlloQuant_output_file_manifest_v7r3.xlsx
+++ b/docs/AlloQuant_output_file_manifest_v7r3.xlsx
@@ -510,14 +510,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reference run: CSK-SRC dimer scan, 260718 rerun (AF3-complete)   |   generated 2026-07-30</t>
+          <t>Reference run: CSK-SRC dimer scan, 260718 rerun (AF3-complete)   |   generated 2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>- AlloQuant is a two-module pipeline. Module 1 (structural extraction) writes the run-root files below; Module 2 (allostery discovery) writes one plots_and_stats_{KINASE}_{METHOD}/ folder per analysed kinase.</t>
+          <t>- AlloQuant is a two-module pipeline. Module 1 (structural extraction) writes the run-root files below, except row 1: experiment.csv is the user-supplied design file it reads. Module 2 (allostery discovery) writes one plots_and_stats_{KINASE}_{METHOD}/ folder per analysed kinase.</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -607,7 +606,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>User input</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -627,7 +626,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Experiment design table: one row per dimer condition (chain_a, condition_a, chain_b, ptm_b, condition_b). Defines the systems built and analysed.</t>
+          <t>User-supplied experimental design metadata: one row per dimer condition (chain_a, condition_a, chain_b, ptm_b, condition_b). Read by the pipeline to define the systems built and analysed; it is not written by AlloQuant and is excluded from run archiving.</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">

</xml_diff>